<commit_message>
[test] 10주차 TC, BTL, 이슈전달 문서
</commit_message>
<xml_diff>
--- a/Assets/Planning/QA/Revenger_BTL.xlsx
+++ b/Assets/Planning/QA/Revenger_BTL.xlsx
@@ -22,17 +22,17 @@
   <calcPr/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:revision xmlns:pm="smNativeData" day="1763127194" val="1228" rev="124" revOS="4" revMin="124" revMax="0"/>
-      <pm:docPrefs xmlns:pm="smNativeData" id="1763127194" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
-      <pm:compatibility xmlns:pm="smNativeData" id="1763127194" overlapCells="1"/>
-      <pm:defCurrency xmlns:pm="smNativeData" id="1763127194"/>
+      <pm:revision xmlns:pm="smNativeData" day="1763650637" val="1228" rev="124" revOS="4" revMin="124" revMax="0"/>
+      <pm:docPrefs xmlns:pm="smNativeData" id="1763650637" fixedDigits="0" showNotice="1" showFrameBounds="1" autoChart="1" recalcOnPrint="1" recalcOnCopy="1" finalRounding="1" compatTextArt="1" tab="567" useDefinedPrintRange="1" printArea="currentSheet"/>
+      <pm:compatibility xmlns:pm="smNativeData" id="1763650637" overlapCells="1"/>
+      <pm:defCurrency xmlns:pm="smNativeData" id="1763650637"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="418" uniqueCount="73">
   <si>
     <t>Date</t>
   </si>
@@ -59,6 +59,9 @@
   </si>
   <si>
     <t>Charger</t>
+  </si>
+  <si>
+    <t>더미</t>
   </si>
   <si>
     <t>Product</t>
@@ -106,7 +109,7 @@
     <t>Issue No.</t>
   </si>
   <si>
-    <t>dd2a22d - 21</t>
+    <t>473a238 - 25</t>
   </si>
   <si>
     <t>TD</t>
@@ -160,22 +163,22 @@
     <t>Category</t>
   </si>
   <si>
-    <t>Scripts</t>
+    <t>Design</t>
   </si>
   <si>
     <t>Charger</t>
   </si>
   <si>
-    <t>이민기</t>
+    <t>엄기영</t>
   </si>
   <si>
     <t>Detail</t>
   </si>
   <si>
-    <t>문이 열리지 않고 테드리만 열리는 버그</t>
+    <t>외부 건물 기둥에 콜리전 누락</t>
   </si>
   <si>
-    <t xml:space="preserve">문이 제대로 열리지 않고 테두리로 추정되는 오브젝트만 열려 진행이 불가함. </t>
+    <t>건물 기둥에 히트박스가 존재하지 않음</t>
   </si>
   <si>
     <t>Replay</t>
@@ -184,64 +187,67 @@
     <t>Comment</t>
   </si>
   <si>
-    <t>문 프리팹에 문제가 있던 것으로 판단</t>
+    <t>기둥에 히트박스 추가 요청</t>
   </si>
   <si>
     <t>Steel shot</t>
   </si>
   <si>
-    <t>dd2a22d - 22</t>
+    <t>473a238 - 26</t>
+  </si>
+  <si>
+    <t>Scripts</t>
+  </si>
+  <si>
+    <t>이민기</t>
+  </si>
+  <si>
+    <t>(디버그) 노클립 이후 퍼즐 시퀀스 버그</t>
+  </si>
+  <si>
+    <t>노클립사용 이후 퍼즐 이용시 하수구 퍼즐 시퀀스만 들어가지는 버그</t>
+  </si>
+  <si>
+    <t>상호작용이 해당 퍼즐로 목표가 잡혀있는데 다른곳으로 강제 이동되어 생긴 문제 (급히 수정됨)</t>
+  </si>
+  <si>
+    <t>473a238 - 27</t>
+  </si>
+  <si>
+    <t>갑자기 모든 경비원에게 발각 버그</t>
+  </si>
+  <si>
+    <t>뛰어다니면 가끔씩 모든 경비병에게 발각되는 버그가 있음</t>
+  </si>
+  <si>
+    <t>경비병에게 발각되는 기준을 확실히 알기가 어려워 원인 파악이 힘듬</t>
+  </si>
+  <si>
+    <t>473a238 - 28</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dress/Guest 퍼즐 클리어후에도 다이얼 UI 접근 가능 </t>
+  </si>
+  <si>
+    <t>Dress/Guest 퍼즐 클리어후에도 다이얼 UI 접근이 가능한 버그</t>
+  </si>
+  <si>
+    <t>의도 된것인지는 아직 파악이 안됨.</t>
+  </si>
+  <si>
+    <t>473a238 - 29</t>
+  </si>
+  <si>
+    <t>식당 퍼즐 ui 일시정지 UI 꼬임</t>
+  </si>
+  <si>
+    <t>식당 퍼즐 ui가 출력되는 동안 esc를 누를시 ui가 꼬임</t>
+  </si>
+  <si>
+    <t>퍼즐 Ui와 일시정지 Ui의 배치를 다시 해야함</t>
   </si>
   <si>
     <t>Yes</t>
-  </si>
-  <si>
-    <t>Home → Outside 씬 이동 버그</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Home씬에서 미션을 시작했을 시 야외 맵으로 이동시 플레이어 프리팹이 제대로 생성되지 않는 버그 발생</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 플레이어 프리팹이 씬으로 제대로 이송되도록 확인해야함 (급히 수정됨)</t>
-  </si>
-  <si>
-    <t>dd2a22d - 23</t>
-  </si>
-  <si>
-    <t>라이터 아이템 획득 불가 버그</t>
-  </si>
-  <si>
-    <t>drawing 퍼즐을 진행하기 위한 라이터 오브젝트(아이템)가 상호작용 키로 집어지지 않음</t>
-  </si>
-  <si>
-    <t>해당 라이터 오브젝트의 레이어, 혹은 코드 충돌이 있는 것으로 판단</t>
-  </si>
-  <si>
-    <t>Villan - A  공격시 동작 무한 반복 버그</t>
-  </si>
-  <si>
-    <t>무기를 꺼내고 Villan - A를 공격시 좌클릭을 연타할시 캐릭터의 공격 애니메이션이 반복되는 버그가 발생함.</t>
-  </si>
-  <si>
-    <t>주인공의 공격시스템, 애니메이션(animator) 파일을 검포해볼 필요가 있음.</t>
-  </si>
-  <si>
-    <t>7e18ef3 - 16</t>
-  </si>
-  <si>
-    <t>Design</t>
-  </si>
-  <si>
-    <t>엄기영</t>
-  </si>
-  <si>
-    <t>경비원이 문 안으로 들어오지 못하는 버그</t>
-  </si>
-  <si>
-    <t>방 사이간 이어지는 문을 통해 경비원이 주인공을 잡기 위해 들어오지 못하는 버그</t>
-  </si>
-  <si>
-    <t>문 사이에도 이동 범위를 따로 추가해 넣을 필요가 있음</t>
   </si>
   <si>
     <t>7e18ef3</t>
@@ -273,7 +279,7 @@
       <sz val="11"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" ulstyle="none" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="Times New Roman" sz="220" lang="default"/>
             <pm:ea face="SimSun" sz="220" lang="default"/>
@@ -288,7 +294,7 @@
       <sz val="10"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" ulstyle="none" kern="1">
             <pm:latin face="Arial" sz="200" lang="default"/>
             <pm:cs face="Times New Roman" sz="200" lang="default"/>
             <pm:ea face="SimSun" sz="200" lang="default"/>
@@ -304,7 +310,7 @@
       <sz val="9"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" ulstyle="none" kern="1">
             <pm:latin face="맑은 고딕" sz="180" lang="default"/>
             <pm:cs face="Times New Roman" sz="180" lang="default"/>
             <pm:ea face="SimSun" sz="180" lang="default"/>
@@ -321,7 +327,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="Times New Roman" sz="220" lang="default"/>
             <pm:ea face="SimSun" sz="220" lang="default"/>
@@ -336,7 +342,7 @@
       <sz val="9"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="180" lang="default"/>
             <pm:cs face="Times New Roman" sz="180" lang="default"/>
             <pm:ea face="SimSun" sz="180" lang="default"/>
@@ -352,7 +358,7 @@
       <sz val="8"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="160" lang="default" weight="bold"/>
             <pm:cs face="Times New Roman" sz="160" lang="default" weight="bold"/>
             <pm:ea face="SimSun" sz="160" lang="default" weight="bold"/>
@@ -368,7 +374,7 @@
       <sz val="12"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="240" lang="default" weight="bold"/>
             <pm:cs face="Times New Roman" sz="240" lang="default" weight="bold"/>
             <pm:ea face="SimSun" sz="240" lang="default" weight="bold"/>
@@ -385,7 +391,7 @@
       <sz val="6"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" ulstyle="none" kern="1">
             <pm:latin face="맑은 고딕" sz="120" lang="default" weight="bold"/>
             <pm:cs face="Times New Roman" sz="120" lang="default" weight="bold"/>
             <pm:ea face="SimSun" sz="120" lang="default" weight="bold"/>
@@ -401,7 +407,7 @@
       <sz val="6"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" ulstyle="none" kern="1">
             <pm:latin face="맑은 고딕" sz="120" lang="default"/>
             <pm:cs face="Times New Roman" sz="120" lang="default"/>
             <pm:ea face="SimSun" sz="120" lang="default"/>
@@ -417,7 +423,7 @@
       <sz val="9"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="180" lang="default" weight="bold"/>
             <pm:cs face="Times New Roman" sz="180" lang="default" weight="bold"/>
             <pm:ea face="SimSun" sz="180" lang="default" weight="bold"/>
@@ -432,7 +438,7 @@
       <sz val="8"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" ulstyle="none" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" ulstyle="none" kern="1">
             <pm:latin face="Calibri" sz="160" lang="default"/>
             <pm:cs face="Times New Roman" sz="160" lang="default"/>
             <pm:ea face="SimSun" sz="160" lang="default"/>
@@ -449,61 +455,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
-            <pm:latin face="맑은 고딕" sz="220" lang="default"/>
-            <pm:cs face="Times New Roman" sz="220" lang="default"/>
-            <pm:ea face="SimSun" sz="220" lang="default"/>
-            <hyperlink type="5" url="" location="'1'!A1" text="'1'!A1"/>
-          </pm:charSpec>
-        </ext>
-      </extLst>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <charset val="129"/>
-      <family val="3"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
-            <pm:latin face="맑은 고딕" sz="220" lang="default"/>
-            <pm:cs face="맑은 고딕" sz="220" lang="default"/>
-            <pm:ea face="맑은 고딕" sz="220" lang="default"/>
-            <hyperlink type="5" url="" location="'6'!A1" text=""/>
-          </pm:charSpec>
-        </ext>
-      </extLst>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <charset val="129"/>
-      <family val="3"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
-            <pm:latin face="맑은 고딕" sz="220" lang="default"/>
-            <pm:cs face="맑은 고딕" sz="220" lang="default"/>
-            <pm:ea face="맑은 고딕" sz="220" lang="default"/>
-            <hyperlink type="5" url="" location="'7'!A1" text=""/>
-          </pm:charSpec>
-        </ext>
-      </extLst>
-    </font>
-    <font>
-      <name val="맑은 고딕"/>
-      <charset val="129"/>
-      <family val="3"/>
-      <color rgb="FF0000FF"/>
-      <sz val="11"/>
-      <u val="single"/>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="맑은 고딕" sz="220" lang="default"/>
             <pm:ea face="맑은 고딕" sz="220" lang="default"/>
@@ -521,7 +473,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="맑은 고딕" sz="220" lang="default"/>
             <pm:ea face="맑은 고딕" sz="220" lang="default"/>
@@ -539,7 +491,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="맑은 고딕" sz="220" lang="default"/>
             <pm:ea face="맑은 고딕" sz="220" lang="default"/>
@@ -557,7 +509,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="맑은 고딕" sz="220" lang="default"/>
             <pm:ea face="맑은 고딕" sz="220" lang="default"/>
@@ -575,7 +527,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="맑은 고딕" sz="220" lang="default"/>
             <pm:ea face="맑은 고딕" sz="220" lang="default"/>
@@ -593,7 +545,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="맑은 고딕" sz="220" lang="default"/>
             <pm:ea face="맑은 고딕" sz="220" lang="default"/>
@@ -611,7 +563,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="맑은 고딕" sz="220" lang="default"/>
             <pm:ea face="맑은 고딕" sz="220" lang="default"/>
@@ -629,7 +581,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="맑은 고딕" sz="220" lang="default"/>
             <pm:ea face="맑은 고딕" sz="220" lang="default"/>
@@ -647,7 +599,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="맑은 고딕" sz="220" lang="default"/>
             <pm:ea face="맑은 고딕" sz="220" lang="default"/>
@@ -665,7 +617,7 @@
       <u val="single"/>
       <extLst>
         <ext uri="smNativeData">
-          <pm:charSpec xmlns:pm="smNativeData" id="1763127194" fgClr="0000FF" ulstyle="single" kern="1">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
             <pm:latin face="맑은 고딕" sz="220" lang="default"/>
             <pm:cs face="맑은 고딕" sz="220" lang="default"/>
             <pm:ea face="맑은 고딕" sz="220" lang="default"/>
@@ -674,8 +626,62 @@
         </ext>
       </extLst>
     </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
+            <pm:latin face="맑은 고딕" sz="220" lang="default"/>
+            <pm:cs face="맑은 고딕" sz="220" lang="default"/>
+            <pm:ea face="맑은 고딕" sz="220" lang="default"/>
+            <hyperlink type="5" url="" location="'17'!A1" text=""/>
+          </pm:charSpec>
+        </ext>
+      </extLst>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
+            <pm:latin face="맑은 고딕" sz="220" lang="default"/>
+            <pm:cs face="맑은 고딕" sz="220" lang="default"/>
+            <pm:ea face="맑은 고딕" sz="220" lang="default"/>
+            <hyperlink type="5" url="" location="'18'!A1" text=""/>
+          </pm:charSpec>
+        </ext>
+      </extLst>
+    </font>
+    <font>
+      <name val="맑은 고딕"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <extLst>
+        <ext uri="smNativeData">
+          <pm:charSpec xmlns:pm="smNativeData" id="1763650637" fgClr="0000FF" ulstyle="single" kern="1">
+            <pm:latin face="맑은 고딕" sz="220" lang="default"/>
+            <pm:cs face="맑은 고딕" sz="220" lang="default"/>
+            <pm:ea face="맑은 고딕" sz="220" lang="default"/>
+            <hyperlink type="5" url="" location="'19'!A1" text=""/>
+          </pm:charSpec>
+        </ext>
+      </extLst>
+    </font>
   </fonts>
-  <fills count="17">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -688,7 +694,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1763127194" type="1" fgLvl="100" fgClr="00BFBFBF" bgLvl="0" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1763650637" type="1" fgLvl="100" fgClr="00BFBFBF" bgLvl="0" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -702,7 +708,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1763127194" type="1" fgLvl="100" fgClr="00D8D8D8" bgLvl="0" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1763650637" type="1" fgLvl="100" fgClr="00D8D8D8" bgLvl="0" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -713,7 +719,7 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1763127194" type="1" fgLvl="100" fgClr="00BFBFBF" bgLvl="0" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1763650637" type="1" fgLvl="100" fgClr="00BFBFBF" bgLvl="0" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
@@ -751,24 +757,13 @@
         <bgColor rgb="FFFFFFFF"/>
         <extLst>
           <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1763127194" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
-          </ext>
-        </extLst>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFD8D8D8"/>
-        <bgColor rgb="FFFFFFFF"/>
-        <extLst>
-          <ext uri="smNativeData">
-            <pm:shade xmlns:pm="smNativeData" id="1763127194" type="1" fgLvl="100" fgClr="00D8D8D8" bgLvl="0" bgClr="00000000"/>
+            <pm:shade xmlns:pm="smNativeData" id="1763650637" type="1" fgLvl="100" fgClr="00FFFFFF" bgLvl="100" bgClr="00000000"/>
           </ext>
         </extLst>
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="15">
     <border>
       <left style="none">
         <color rgb="FF000000"/>
@@ -784,7 +779,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194"/>
+          <pm:border xmlns:pm="smNativeData" id="1763650637"/>
         </ext>
       </extLst>
     </border>
@@ -803,7 +798,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194"/>
+          <pm:border xmlns:pm="smNativeData" id="1763650637"/>
         </ext>
       </extLst>
     </border>
@@ -822,7 +817,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -846,7 +841,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -870,7 +865,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -894,7 +889,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -915,7 +910,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -937,7 +932,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
         </ext>
@@ -958,7 +953,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -980,7 +975,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -1002,7 +997,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -1024,7 +1019,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="left" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1047,7 +1042,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
           </pm:border>
@@ -1069,7 +1064,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194">
+          <pm:border xmlns:pm="smNativeData" id="1763650637">
             <pm:line position="top" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="bottom" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
             <pm:line position="right" type="1" style="0" width="20" dist="20" width2="20" rgb="000000"/>
@@ -1092,26 +1087,7 @@
       </bottom>
       <extLst>
         <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194"/>
-        </ext>
-      </extLst>
-    </border>
-    <border>
-      <left style="none">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="none">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="none">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom style="none">
-        <color rgb="FF000000"/>
-      </bottom>
-      <extLst>
-        <ext uri="smNativeData">
-          <pm:border xmlns:pm="smNativeData" id="1763127194"/>
+          <pm:border xmlns:pm="smNativeData" id="1763650637"/>
         </ext>
       </extLst>
     </border>
@@ -1212,14 +1188,14 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1245,7 +1221,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="20" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1254,7 +1230,7 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="23" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1265,10 +1241,10 @@
   <tableStyles count="0"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:charStyles xmlns:pm="smNativeData" id="1763127194" count="1">
+      <pm:charStyles xmlns:pm="smNativeData" id="1763650637" count="1">
         <pm:charStyle name="보통" fontId="0" Id="1"/>
       </pm:charStyles>
-      <pm:colors xmlns:pm="smNativeData" id="1763127194" count="2">
+      <pm:colors xmlns:pm="smNativeData" id="1763650637" count="2">
         <pm:color name="색: 24" rgb="D8D8D8"/>
         <pm:color name="색: 25" rgb="BFBFBF"/>
       </pm:colors>
@@ -1282,15 +1258,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>95250</xdr:colOff>
+      <xdr:colOff>0</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>96520</xdr:rowOff>
+      <xdr:rowOff>37465</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>368300</xdr:colOff>
+      <xdr:colOff>666115</xdr:colOff>
       <xdr:row>35</xdr:row>
-      <xdr:rowOff>109855</xdr:rowOff>
+      <xdr:rowOff>64770</xdr:rowOff>
     </xdr:to>
     <xdr:pic macro="">
       <xdr:nvPicPr>
@@ -1299,7 +1275,7 @@
           <a:picLocks noChangeAspect="1"/>
           <a:extLst>
             <a:ext uri="smNativeData">
-              <pm:smNativeData xmlns:pm="smNativeData" val="SMDATA_15_mi8XaRMAAAAlAAAAEQAAAK8BAAAAkAAAAEgAAACQAAAASAAAAAAAAAAAAAAAAAAAAAEAAABQAAAAAAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8CAAAAjAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAZAAAAAEAAABAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAFAAAADwAAAAAAAAAAAAAAAAAAAAUAAAAAQAAABQAAAAUAAAAFAAAAAEAAAAAAAAAZAAAAGQAAAAAAAAAZAAAAGQAAAAVAAAAYAAAAAAAAAAAAAAADwAAACADAAAAAAAAAAAAAAEAAACgMgAAVgcAAKr4//8BAAAAf39/AAEAAABkAAAAAAAAABQAAABAHwAAAAAAACYAAAAAAAAAwOD//wAAAAAmAAAAZAAAABYAAABMAAAAAAAAAAAAAAAEAAAAAAAAAAEAAAB/f38AAAAAACgAAAAoAAAAZAAAAGQAAAAAAAAAzMzMAAAAAABQAAAAUAAAAGQAAABkAAAAAAAAAAcAAAA4AAAAAAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABkAAAAZAAAAAAAAAAjAAAABAAAAGQAAAAXAAAAFAAAAAAAAAAAAAAA/38AAP9/AAAAAAAACQAAAAQAAADGQt+GHgAAAGgAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABAnAAAQJwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAUAAAAAAAAAMDA/wAAAAAAZAAAADIAAAAAAAAAZAAAAAAAAAB/f38ACgAAACIAAAAYAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAJAAAACQAAAAAAAAABwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAH9/fwAlAAAAWAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAPwAAAAAAAACghgEAAAAAAAAAAAAAAAAADAAAAAEAAAAAAAAAAAAAAAAAAAAhAAAAMAAAACwAAAAVAAAAAAAAAG4BkAAjAAAACQAAAKEBLgKWAAAAXyEAABYnAABhFwAAAAAAAA=="/>
+              <pm:smNativeData xmlns:pm="smNativeData" val="SMDATA_15_TSwfaRMAAAAlAAAAEQAAAK8BAAAAkAAAAEgAAACQAAAASAAAAAAAAAAAAAAAAAAAAAEAAABQAAAAAAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8CAAAAjAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAZAAAAAEAAABAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAFAAAADwAAAAAAAAAAAAAAAAAAAAUAAAAAQAAABQAAAAUAAAAFAAAAAEAAAAAAAAAZAAAAGQAAAAAAAAAZAAAAGQAAAAVAAAAYAAAAAAAAAAAAAAADwAAACADAAAAAAAAAAAAAAEAAACgMgAAVgcAAKr4//8BAAAAf39/AAEAAABkAAAAAAAAABQAAABAHwAAAAAAACYAAAAAAAAAwOD//wAAAAAmAAAAZAAAABYAAABMAAAAAAAAAAAAAAAEAAAAAAAAAAEAAAB/f38AAAAAACgAAAAoAAAAZAAAAGQAAAAAAAAAzMzMAAAAAABQAAAAUAAAAGQAAABkAAAAAAAAAAcAAAA4AAAAAAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABkAAAAZAAAAAAAAAAjAAAABAAAAGQAAAAXAAAAFAAAAAAAAAAAAAAA/38AAP9/AAAAAAAACQAAAAQAAAAYAgAAHgAAAGgAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABAnAAAQJwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAUAAAAAAAAAMDA/wAAAAAAZAAAADIAAAAAAAAAZAAAAAAAAAB/f38ACgAAACIAAAAYAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAJAAAACQAAAAAAAAABwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAH9/fwAlAAAAWAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAPwAAAAAAAACghgEAAAAAAAAAAAAAAAAADAAAAAEAAAAAAAAAAAAAAAAAAAAhAAAAMAAAACwAAAAVAAAAAAAAAI4AAAAjAAAACQAAAPUA8gMAAAAAAiEAAIEpAAB3FwAAAAAAAA=="/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPicPr>
@@ -1312,8 +1288,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="95250" y="5424805"/>
-          <a:ext cx="6353810" cy="3800475"/>
+          <a:off x="0" y="5365750"/>
+          <a:ext cx="6746875" cy="3814445"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1338,172 +1314,6 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>96520</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>528320</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>116205</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic macro="">
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="그림1"/>
-        <xdr:cNvPicPr>
-          <a:extLst>
-            <a:ext uri="smNativeData">
-              <pm:smNativeData xmlns:pm="smNativeData" val="SMDATA_15_mi8XaRMAAAAlAAAAEQAAAI8BAAAAkAAAAEgAAACQAAAASAAAAAAAAAAAAAAAAAAAAAEAAABQAAAAAAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8CAAAAjAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAZAAAAAEAAABAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAFAAAADwAAAAAAAAAAAAAAAAAAAAUAAAAAQAAABQAAAAUAAAAFAAAAAEAAAAAAAAAZAAAAGQAAAAAAAAAZAAAAGQAAAAVAAAAYAAAAAAAAAAAAAAADwAAACADAAAAAAAAAAAAAAEAAACgMgAAVgcAAKr4//8BAAAAf39/AAEAAABkAAAAAAAAABQAAABAHwAAAAAAACYAAAAAAAAAwOD//wAAAAAmAAAAZAAAABYAAABMAAAAAAAAAAAAAAAEAAAAAAAAAAEAAAB/f38AAAAAACgAAAAoAAAAZAAAAGQAAAAAAAAAzMzMAAAAAABQAAAAUAAAAGQAAABkAAAAAAAAAAcAAAA4AAAAAAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABkAAAAZAAAAAAAAAAjAAAABAAAAGQAAAAXAAAAFAAAAAAAAAAAAAAA/38AAP9/AAAAAAAACQAAAAQAAAAABgAAHgAAAGgAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABAnAAAQJwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAUAAAAAAAAAMDA/wAAAAAAZAAAADIAAAAAAAAAZAAAAAAAAAB/f38ACgAAACIAAAAYAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAJAAAACQAAAAAAAAABwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAH9/fwAlAAAAWAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAPwAAAAAAAACghgEAAAAAAAAAAAAAAAAADAAAAAEAAAAAAAAAAAAAAAAAAAAhAAAAMAAAACwAAAAVAAAAAAAAAG4BAAAmAAAACQAAALcBIQMAAAAAXyEAAKgoAABpHAAAAAAAAA=="/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="5424805"/>
-          <a:ext cx="6609080" cy="4618355"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-          <a:headEnd type="none" w="med" len="med"/>
-          <a:tailEnd type="none" w="med" len="med"/>
-        </a:ln>
-        <a:effectLst/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>29210</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>4445</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic macro="">
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="그림1"/>
-        <xdr:cNvPicPr>
-          <a:extLst>
-            <a:ext uri="smNativeData">
-              <pm:smNativeData xmlns:pm="smNativeData" val="SMDATA_15_mi8XaRMAAAAlAAAAEQAAAI8BAAAAkAAAAEgAAACQAAAASAAAAAAAAAAAAAAAAAAAAAEAAABQAAAAAAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8CAAAAjAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAZAAAAAEAAABAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAFAAAADwAAAAAAAAAAAAAAAAAAAAUAAAAAQAAABQAAAAUAAAAFAAAAAEAAAAAAAAAZAAAAGQAAAAAAAAAZAAAAGQAAAAVAAAAYAAAAAAAAAAAAAAADwAAACADAAAAAAAAAAAAAAEAAACgMgAAVgcAAKr4//8BAAAAf39/AAEAAABkAAAAAAAAABQAAABAHwAAAAAAACYAAAAAAAAAwOD//wAAAAAmAAAAZAAAABYAAABMAAAAAAAAAAAAAAAEAAAAAAAAAAEAAAB/f38AAAAAACgAAAAoAAAAZAAAAGQAAAAAAAAAzMzMAAAAAABQAAAAUAAAAGQAAABkAAAAAAAAAAcAAAA4AAAAAAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABkAAAAZAAAAAAAAAAjAAAABAAAAGQAAAAXAAAAFAAAAAAAAAAAAAAA/38AAP9/AAAAAAAACQAAAAQAAAAAAAAAHgAAAGgAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABAnAAAQJwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAUAAAAAAAAAMDA/wAAAAAAZAAAADIAAAAAAAAAZAAAAAAAAAB/f38ACgAAACIAAAAYAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAJAAAACQAAAAAAAAABwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAH9/fwAlAAAAWAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAPwAAAAAAAACghgEAAAAAAAAAAAAAAAAADAAAAAEAAAAAAAAAAAAAAAAAAAAhAAAAMAAAACwAAAAVAAAAAAAAAG4AAAAfAAAACgAAAAAABwAAAAAA9SAAAJcpAAB2EAAAAAAAAA=="/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="0" y="5357495"/>
-          <a:ext cx="6760845" cy="2675890"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-          <a:headEnd type="none" w="med" len="med"/>
-          <a:tailEnd type="none" w="med" len="med"/>
-        </a:ln>
-        <a:effectLst/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>635</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>135255</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>654685</xdr:colOff>
-      <xdr:row>35</xdr:row>
-      <xdr:rowOff>203200</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic macro="">
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="그림1"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-          <a:extLst>
-            <a:ext uri="smNativeData">
-              <pm:smNativeData xmlns:pm="smNativeData" val="SMDATA_15_mi8XaRMAAAAlAAAAEQAAAK8BAAAAkAAAAEgAAACQAAAASAAAAAAAAAAAAAAAAAAAAAEAAABQAAAAAAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8CAAAAjAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAZAAAAAEAAABAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAFAAAADwAAAAAAAAAAAAAAAAAAAAUAAAAAQAAABQAAAAUAAAAFAAAAAEAAAAAAAAAZAAAAGQAAAAAAAAAZAAAAGQAAAAVAAAAYAAAAAAAAAAAAAAADwAAACADAAAAAAAAAAAAAAEAAACgMgAAVgcAAKr4//8BAAAAf39/AAEAAABkAAAAAAAAABQAAABAHwAAAAAAACYAAAAAAAAAwOD//wAAAAAmAAAAZAAAABYAAABMAAAAAAAAAAAAAAAEAAAAAAAAAAEAAAB/f38AAAAAACgAAAAoAAAAZAAAAGQAAAAAAAAAzMzMAAAAAABQAAAAUAAAAGQAAABkAAAAAAAAAAcAAAA4AAAAAAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABkAAAAZAAAAAAAAAAjAAAABAAAAGQAAAAXAAAAFAAAAAAAAAAAAAAA/38AAP9/AAAAAAAACQAAAAQAAAAAAAAAHgAAAGgAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABAnAAAQJwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAUAAAAAAAAAMDA/wAAAAAAZAAAADIAAAAAAAAAZAAAAAAAAAB/f38ACgAAACIAAAAYAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAJAAAACQAAAAAAAAABwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAH9/fwAlAAAAWAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAPwAAAAAAAACghgEAAAAAAAAAAAAAAAAADAAAAAEAAAAAAAAAAAAAAAAAAAAhAAAAMAAAACwAAAAVAAAAAAAAAAACAQAjAAAACQAAAAED4AMBAAAAnCEAAG4pAAC3FwAAAAAAAA=="/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="635" y="5463540"/>
-          <a:ext cx="6734810" cy="3855085"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:prstDash val="solid"/>
-          <a:headEnd type="none" w="med" len="med"/>
-          <a:tailEnd type="none" w="med" len="med"/>
-        </a:ln>
-        <a:effectLst/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
       <xdr:colOff>9525</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>241300</xdr:rowOff>
@@ -1521,7 +1331,7 @@
           <a:picLocks noChangeAspect="1"/>
           <a:extLst>
             <a:ext uri="smNativeData">
-              <pm:smNativeData xmlns:pm="smNativeData" val="SMDATA_15_mi8XaRMAAAAlAAAAEQAAAK8BAAAAkAAAAEgAAACQAAAASAAAAAAAAAAAAAAAAAAAAAEAAABQAAAAAAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8CAAAAjAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAZAAAAAEAAABAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAFAAAADwAAAAAAAAAAAAAAAAAAAAUAAAAAQAAABQAAAAUAAAAFAAAAAEAAAAAAAAAZAAAAGQAAAAAAAAAZAAAAGQAAAAVAAAAYAAAAAAAAAAAAAAADwAAACADAAAAAAAAAAAAAAEAAACgMgAAVgcAAKr4//8BAAAAf39/AAEAAABkAAAAAAAAABQAAABAHwAAAAAAACYAAAAAAAAAwOD//wAAAAAmAAAAZAAAABYAAABMAAAAAAAAAAAAAAAEAAAAAAAAAAEAAAB/f38AAAAAACgAAAAoAAAAZAAAAGQAAAAAAAAAzMzMAAAAAABQAAAAUAAAAGQAAABkAAAAAAAAAAcAAAA4AAAAAAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABkAAAAZAAAAAAAAAAjAAAABAAAAGQAAAAXAAAAFAAAAAAAAAAAAAAA/38AAP9/AAAAAAAACQAAAAQAAAAAAAAAHgAAAGgAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABAnAAAQJwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAUAAAAAAAAAMDA/wAAAAAAZAAAADIAAAAAAAAAZAAAAAAAAAB/f38ACgAAACIAAAAYAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAJAAAACQAAAAAAAAABwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAH9/fwAlAAAAWAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAPwAAAAAAAACghgEAAAAAAAAAAAAAAAAADAAAAAEAAAAAAAAAAAAAAAAAAAAhAAAAMAAAACwAAAAWAAAAAAAAAJEDDgAlAAAACQAAACgDawMPAAAA7SMAAOYoAADKGAAAAAAAAA=="/>
+              <pm:smNativeData xmlns:pm="smNativeData" val="SMDATA_15_TSwfaRMAAAAlAAAAEQAAAK8BAAAAkAAAAEgAAACQAAAASAAAAAAAAAAAAAAAAAAAAAEAAABQAAAAAAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8AAAAAAADgPwAAAAAAAOA/AAAAAAAA4D8CAAAAjAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAZAAAAAEAAABAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAFAAAADwAAAAAAAAAAAAAAAAAAAAUAAAAAQAAABQAAAAUAAAAFAAAAAEAAAAAAAAAZAAAAGQAAAAAAAAAZAAAAGQAAAAVAAAAYAAAAAAAAAAAAAAADwAAACADAAAAAAAAAAAAAAEAAACgMgAAVgcAAKr4//8BAAAAf39/AAEAAABkAAAAAAAAABQAAABAHwAAAAAAACYAAAAAAAAAwOD//wAAAAAmAAAAZAAAABYAAABMAAAAAAAAAAAAAAAEAAAAAAAAAAEAAAB/f38AAAAAACgAAAAoAAAAZAAAAGQAAAAAAAAAzMzMAAAAAABQAAAAUAAAAGQAAABkAAAAAAAAAAcAAAA4AAAAAAAAAAAAAAAAAAAA////AAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABkAAAAZAAAAAAAAAAjAAAABAAAAGQAAAAXAAAAFAAAAAAAAAAAAAAA/38AAP9/AAAAAAAACQAAAAQAAAAAAAAAHgAAAGgAAAAAAAAAAAAAAAAAAAAAAAAAAAAAABAnAAAQJwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAUAAAAAAAAAMDA/wAAAAAAZAAAADIAAAAAAAAAZAAAAAAAAAB/f38ACgAAACIAAAAYAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAJAAAACQAAAAAAAAABwAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAH9/fwAlAAAAWAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAAPwAAAAAAAACghgEAAAAAAAAAAAAAAAAADAAAAAEAAAAAAAAAAAAAAAAAAAAhAAAAMAAAACwAAAAWAAAAAAAAAJEDDgAlAAAACQAAACgDawMPAAAA7SMAAOYoAADKGAAAAAAAAA=="/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPicPr>
@@ -1811,7 +1621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <dimension ref="A1:H26"/>
+  <dimension ref="A1:H30"/>
   <sheetFormatPr defaultRowHeight="21"/>
   <cols>
     <col min="1" max="1" width="7.297521" customWidth="1" style="7"/>
@@ -1829,7 +1639,7 @@
       </c>
       <c r="G1" s="14">
         <f aca="1">TODAY()</f>
-        <v>45975</v>
+        <v>45981</v>
       </c>
       <c r="H1" s="14"/>
     </row>
@@ -1872,28 +1682,28 @@
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="38" t="n">
+      <c r="A4" s="35" t="n">
         <v>12</v>
       </c>
       <c r="B4" s="9">
         <f>'12'!C4</f>
-        <v>45975</v>
+        <v>45981</v>
       </c>
       <c r="C4" s="8" t="str">
         <f>'12'!C3</f>
-        <v>dd2a22d - 21</v>
+        <v>473a238 - 25</v>
       </c>
       <c r="D4" s="8" t="str">
         <f>'12'!C9</f>
-        <v>Scripts</v>
+        <v>Design</v>
       </c>
       <c r="E4" s="8" t="str">
         <f>'12'!C5</f>
-        <v>High</v>
+        <v>Low</v>
       </c>
       <c r="F4" s="12" t="str">
         <f>'12'!C12</f>
-        <v>문이 열리지 않고 테드리만 열리는 버그</v>
+        <v>외부 건물 기둥에 콜리전 누락</v>
       </c>
       <c r="G4" s="8" t="str">
         <f>'12'!H4</f>
@@ -1901,20 +1711,20 @@
       </c>
       <c r="H4" s="8" t="str">
         <f>'12'!H9</f>
-        <v>이민기</v>
+        <v>엄기영</v>
       </c>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="39" t="n">
+      <c r="A5" s="36" t="n">
         <v>13</v>
       </c>
       <c r="B5" s="9">
         <f>'13'!C4</f>
-        <v>45975</v>
+        <v>45981</v>
       </c>
       <c r="C5" s="8" t="str">
         <f>'13'!C3</f>
-        <v>dd2a22d - 22</v>
+        <v>473a238 - 26</v>
       </c>
       <c r="D5" s="8" t="str">
         <f>'13'!C9</f>
@@ -1922,11 +1732,11 @@
       </c>
       <c r="E5" s="8" t="str">
         <f>'13'!C5</f>
-        <v>High</v>
+        <v>Mid</v>
       </c>
       <c r="F5" s="12" t="str">
         <f>'13'!C12</f>
-        <v>Home → Outside 씬 이동 버그</v>
+        <v>(디버그) 노클립 이후 퍼즐 시퀀스 버그</v>
       </c>
       <c r="G5" s="8" t="str">
         <f>'12'!H4</f>
@@ -1938,16 +1748,16 @@
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="40" t="n">
+      <c r="A6" s="37" t="n">
         <v>14</v>
       </c>
       <c r="B6" s="9">
         <f>'14'!C4</f>
-        <v>45975</v>
+        <v>45981</v>
       </c>
       <c r="C6" s="8" t="str">
         <f>'14'!C3</f>
-        <v>dd2a22d - 23</v>
+        <v>473a238 - 27</v>
       </c>
       <c r="D6" s="8" t="str">
         <f>'14'!C9</f>
@@ -1959,7 +1769,7 @@
       </c>
       <c r="F6" s="12" t="str">
         <f>'14'!C12</f>
-        <v>라이터 아이템 획득 불가 버그</v>
+        <v>갑자기 모든 경비원에게 발각 버그</v>
       </c>
       <c r="G6" s="8" t="str">
         <f>'12'!H4</f>
@@ -1971,16 +1781,16 @@
       </c>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="41" t="n">
+      <c r="A7" s="38" t="n">
         <v>15</v>
       </c>
       <c r="B7" s="9">
         <f>'15'!C4</f>
-        <v>45975</v>
+        <v>45981</v>
       </c>
       <c r="C7" s="8" t="str">
         <f>'15'!C3</f>
-        <v>dd2a22d - 23</v>
+        <v>473a238 - 28</v>
       </c>
       <c r="D7" s="8" t="str">
         <f>'15'!C9</f>
@@ -1988,11 +1798,11 @@
       </c>
       <c r="E7" s="8" t="str">
         <f>'15'!C5</f>
-        <v>Low</v>
+        <v>Mid</v>
       </c>
       <c r="F7" s="12" t="str">
         <f>'15'!C12</f>
-        <v>Villan - A  공격시 동작 무한 반복 버그</v>
+        <v>Dress/Guest 퍼즐 클리어후에도 다이얼 UI 접근 가능 </v>
       </c>
       <c r="G7" s="8" t="str">
         <f>'12'!H4</f>
@@ -2004,7 +1814,7 @@
       </c>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="42" t="n">
+      <c r="A8" s="39" t="n">
         <v>16</v>
       </c>
       <c r="B8" s="9">
@@ -2013,19 +1823,19 @@
       </c>
       <c r="C8" s="8" t="str">
         <f>'16'!C3</f>
-        <v>7e18ef3 - 16</v>
+        <v>473a238 - 29</v>
       </c>
       <c r="D8" s="8" t="str">
         <f>'16'!C9</f>
-        <v>Design</v>
+        <v>Scripts</v>
       </c>
       <c r="E8" s="8" t="str">
-        <f>'15'!C5</f>
-        <v>Low</v>
+        <f>'16'!C5</f>
+        <v>Mid</v>
       </c>
       <c r="F8" s="12" t="str">
         <f>'16'!C12</f>
-        <v>경비원이 문 안으로 들어오지 못하는 버그</v>
+        <v>식당 퍼즐 ui 일시정지 UI 꼬임</v>
       </c>
       <c r="G8" s="8" t="str">
         <f>'12'!H4</f>
@@ -2033,11 +1843,11 @@
       </c>
       <c r="H8" s="8" t="str">
         <f>'16'!H9</f>
-        <v>엄기영</v>
+        <v>이민기</v>
       </c>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="32"/>
+      <c r="A9" s="8"/>
       <c r="B9" s="9"/>
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
@@ -2047,7 +1857,7 @@
       <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="33"/>
+      <c r="A10" s="8"/>
       <c r="B10" s="9"/>
       <c r="C10" s="8"/>
       <c r="D10" s="8"/>
@@ -2057,17 +1867,17 @@
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="29"/>
+      <c r="A11" s="8"/>
       <c r="B11" s="9"/>
       <c r="C11" s="8"/>
-      <c r="D11" s="9"/>
+      <c r="D11" s="8"/>
       <c r="E11" s="8"/>
       <c r="F11" s="12"/>
       <c r="G11" s="8"/>
-      <c r="H11" s="9"/>
+      <c r="H11" s="8"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="43"/>
+      <c r="A12" s="8"/>
       <c r="B12" s="9"/>
       <c r="C12" s="8"/>
       <c r="D12" s="8"/>
@@ -2077,7 +1887,7 @@
       <c r="H12" s="8"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="34"/>
+      <c r="A13" s="31"/>
       <c r="B13" s="9"/>
       <c r="C13" s="8"/>
       <c r="D13" s="8"/>
@@ -2087,7 +1897,7 @@
       <c r="H13" s="8"/>
     </row>
     <row r="14" spans="1:8">
-      <c r="A14" s="35"/>
+      <c r="A14" s="32"/>
       <c r="B14" s="9"/>
       <c r="C14" s="8"/>
       <c r="D14" s="8"/>
@@ -2097,7 +1907,7 @@
       <c r="H14" s="8"/>
     </row>
     <row r="15" spans="1:8">
-      <c r="A15" s="36"/>
+      <c r="A15" s="33"/>
       <c r="B15" s="9"/>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
@@ -2107,7 +1917,7 @@
       <c r="H15" s="8"/>
     </row>
     <row r="16" spans="1:8">
-      <c r="A16" s="37"/>
+      <c r="A16" s="34"/>
       <c r="B16" s="9"/>
       <c r="C16" s="8"/>
       <c r="D16" s="8"/>
@@ -2207,7 +2017,9 @@
       <c r="H25" s="8"/>
     </row>
     <row r="26" spans="1:8">
-      <c r="A26" s="8"/>
+      <c r="A26" s="8" t="s">
+        <v>9</v>
+      </c>
       <c r="B26" s="9"/>
       <c r="C26" s="8"/>
       <c r="D26" s="8"/>
@@ -2215,6 +2027,138 @@
       <c r="F26" s="12"/>
       <c r="G26" s="8"/>
       <c r="H26" s="8"/>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="41" t="n">
+        <v>17</v>
+      </c>
+      <c r="B27" s="9">
+        <f>'17'!C4</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="8">
+        <f>'17'!C3</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="8">
+        <f>'17'!C9</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="8" t="str">
+        <f>'17'!C5</f>
+        <v>Low</v>
+      </c>
+      <c r="F27" s="12">
+        <f>'17'!C12</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="8" t="str">
+        <f>'12'!H4</f>
+        <v>김사윤</v>
+      </c>
+      <c r="H27" s="8">
+        <f>'17'!H9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" s="42" t="n">
+        <v>18</v>
+      </c>
+      <c r="B28" s="9">
+        <f>'18'!C4</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="8">
+        <f>'18'!C3</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="8">
+        <f>'18'!C9</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="8" t="str">
+        <f>'18'!C5</f>
+        <v>Mid</v>
+      </c>
+      <c r="F28" s="12">
+        <f>'18'!C12</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="8" t="str">
+        <f>'12'!H4</f>
+        <v>김사윤</v>
+      </c>
+      <c r="H28" s="8">
+        <f>'18'!H9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" s="43" t="n">
+        <v>19</v>
+      </c>
+      <c r="B29" s="9">
+        <f>'19'!C4</f>
+        <v>0</v>
+      </c>
+      <c r="C29" s="8">
+        <f>'19'!C3</f>
+        <v>0</v>
+      </c>
+      <c r="D29" s="9">
+        <f>'19'!C9</f>
+        <v>0</v>
+      </c>
+      <c r="E29" s="8" t="str">
+        <f>'19'!C5</f>
+        <v>Low</v>
+      </c>
+      <c r="F29" s="12">
+        <f>'19'!C12</f>
+        <v>0</v>
+      </c>
+      <c r="G29" s="8" t="str">
+        <f>'12'!H4</f>
+        <v>김사윤</v>
+      </c>
+      <c r="H29" s="9">
+        <f>'19'!H9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="40" t="n">
+        <v>20</v>
+      </c>
+      <c r="B30" s="9">
+        <f>'20'!C4</f>
+        <v>0</v>
+      </c>
+      <c r="C30" s="8">
+        <f>'20'!C3</f>
+        <v>0</v>
+      </c>
+      <c r="D30" s="8">
+        <f>'20'!C9</f>
+        <v>0</v>
+      </c>
+      <c r="E30" s="8" t="str">
+        <f>'20'!C5</f>
+        <v>Mid</v>
+      </c>
+      <c r="F30" s="12">
+        <f>'20'!C12</f>
+        <v>0</v>
+      </c>
+      <c r="G30" s="8" t="str">
+        <f>'12'!H4</f>
+        <v>김사윤</v>
+      </c>
+      <c r="H30" s="8">
+        <f>'20'!H9</f>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2227,19 +2171,19 @@
     <hyperlink ref="A6" location="'14'!A1"/>
     <hyperlink ref="A7" location="'15'!A1"/>
     <hyperlink ref="A8" location="'16'!A1"/>
-    <hyperlink ref="A9" location="'6'!A1"/>
-    <hyperlink ref="A10" location="'7'!A1"/>
-    <hyperlink ref="A11" location="'1'!A1"/>
-    <hyperlink ref="A12" location="'20'!A1"/>
     <hyperlink ref="A13" location="'9-2'!A1"/>
     <hyperlink ref="A14" location="'10-1'!A1"/>
     <hyperlink ref="A15" location="'10-2'!A1"/>
     <hyperlink ref="A16" location="'11'!A1"/>
+    <hyperlink ref="A27" location="'17'!A1"/>
+    <hyperlink ref="A28" location="'18'!A1"/>
+    <hyperlink ref="A29" location="'19'!A1"/>
+    <hyperlink ref="A30" location="'20'!A1"/>
   </hyperlinks>
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1763127194" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1763650637" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2248,16 +2192,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763127194" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763650637" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -2277,37 +2221,37 @@
   <sheetData>
     <row r="1" spans="5:19">
       <c r="E1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I1" s="25" t="n">
         <v>45950.9236111111095</v>
       </c>
       <c r="J1" s="25"/>
       <c r="O1" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -2319,24 +2263,24 @@
       <c r="I2" s="13"/>
       <c r="J2" s="13"/>
       <c r="O2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="8"/>
@@ -2348,45 +2292,45 @@
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
       <c r="O3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="26"/>
       <c r="D4" s="27"/>
       <c r="E4" s="28"/>
       <c r="F4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="S4" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -2395,27 +2339,27 @@
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
       <c r="S5" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="7" spans="1:10">
       <c r="A7" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -2429,34 +2373,34 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G9" s="11"/>
       <c r="H9" s="9"/>
@@ -2466,7 +2410,7 @@
     <row r="10" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="11" spans="1:10">
       <c r="A11" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -2480,10 +2424,10 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="11"/>
-      <c r="C12" s="30"/>
+      <c r="C12" s="29"/>
       <c r="D12" s="23"/>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
@@ -2493,7 +2437,7 @@
       <c r="J12" s="24"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="31"/>
+      <c r="A13" s="30"/>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
@@ -2518,7 +2462,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="22"/>
@@ -2556,7 +2500,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="22"/>
@@ -2594,7 +2538,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="22"/>
@@ -2963,7 +2907,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1763127194" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1763650637" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -2972,17 +2916,17 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <drawing r:id="rId1"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763127194" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763650637" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3002,37 +2946,37 @@
   <sheetData>
     <row r="1" spans="5:19">
       <c r="E1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I1" s="25" t="n">
         <v>45975.9236111111095</v>
       </c>
       <c r="J1" s="25"/>
       <c r="O1" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -3044,28 +2988,28 @@
       <c r="I2" s="13"/>
       <c r="J2" s="13"/>
       <c r="O2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
@@ -3075,47 +3019,47 @@
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
       <c r="O3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="26" t="n">
-        <v>45975</v>
+        <v>45981</v>
       </c>
       <c r="D4" s="27"/>
       <c r="E4" s="28"/>
       <c r="F4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="S4" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -3124,27 +3068,27 @@
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="8" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
       <c r="S5" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="7" spans="1:10">
       <c r="A7" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -3158,40 +3102,40 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="9" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G9" s="11"/>
       <c r="H9" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
@@ -3199,7 +3143,7 @@
     <row r="10" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="11" spans="1:10">
       <c r="A11" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -3213,11 +3157,11 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="11"/>
-      <c r="C12" s="30" t="s">
-        <v>46</v>
+      <c r="C12" s="29" t="s">
+        <v>47</v>
       </c>
       <c r="D12" s="23"/>
       <c r="E12" s="23"/>
@@ -3228,8 +3172,8 @@
       <c r="J12" s="24"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="31" t="s">
-        <v>47</v>
+      <c r="A13" s="30" t="s">
+        <v>48</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -3255,7 +3199,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="22"/>
@@ -3293,7 +3237,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="22"/>
@@ -3307,7 +3251,7 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
@@ -3333,7 +3277,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="22"/>
@@ -3702,7 +3646,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1763127194" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1763650637" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -3711,17 +3655,17 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <drawing r:id="rId1"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763127194" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763650637" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -3741,37 +3685,37 @@
   <sheetData>
     <row r="1" spans="5:19">
       <c r="E1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I1" s="25" t="n">
         <v>45975.9236111111095</v>
       </c>
       <c r="J1" s="25"/>
       <c r="O1" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -3783,28 +3727,28 @@
       <c r="I2" s="13"/>
       <c r="J2" s="13"/>
       <c r="O2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
@@ -3814,47 +3758,47 @@
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
       <c r="O3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="26" t="n">
-        <v>45975</v>
+        <v>45981</v>
       </c>
       <c r="D4" s="27"/>
       <c r="E4" s="28"/>
       <c r="F4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="S4" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -3863,27 +3807,27 @@
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="8" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
       <c r="S5" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="7" spans="1:10">
       <c r="A7" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -3897,40 +3841,40 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="9" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="8" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="9" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G9" s="11"/>
       <c r="H9" s="9" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
@@ -3938,7 +3882,7 @@
     <row r="10" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="11" spans="1:10">
       <c r="A11" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -3952,11 +3896,11 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="11"/>
-      <c r="C12" s="30" t="s">
-        <v>54</v>
+      <c r="C12" s="29" t="s">
+        <v>56</v>
       </c>
       <c r="D12" s="23"/>
       <c r="E12" s="23"/>
@@ -3967,8 +3911,8 @@
       <c r="J12" s="24"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="31" t="s">
-        <v>55</v>
+      <c r="A13" s="30" t="s">
+        <v>57</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -3994,7 +3938,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="22"/>
@@ -4032,7 +3976,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="22"/>
@@ -4046,7 +3990,7 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
@@ -4072,7 +4016,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="22"/>
@@ -4441,7 +4385,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1763127194" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1763650637" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -4450,17 +4394,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
-  <drawing r:id="rId1"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763127194" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763650637" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -4480,37 +4423,37 @@
   <sheetData>
     <row r="1" spans="5:19">
       <c r="E1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I1" s="25" t="n">
         <v>45975.9236111111095</v>
       </c>
       <c r="J1" s="25"/>
       <c r="O1" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -4522,28 +4465,28 @@
       <c r="I2" s="13"/>
       <c r="J2" s="13"/>
       <c r="O2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="8" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
@@ -4553,47 +4496,47 @@
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
       <c r="O3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="26" t="n">
-        <v>45975</v>
+        <v>45981</v>
       </c>
       <c r="D4" s="27"/>
       <c r="E4" s="28"/>
       <c r="F4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="S4" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -4602,27 +4545,27 @@
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
       <c r="S5" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="7" spans="1:10">
       <c r="A7" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -4636,40 +4579,40 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="9" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="8" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="9" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G9" s="11"/>
       <c r="H9" s="9" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
@@ -4677,7 +4620,7 @@
     <row r="10" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="11" spans="1:10">
       <c r="A11" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -4691,11 +4634,11 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="11"/>
-      <c r="C12" s="30" t="s">
-        <v>58</v>
+      <c r="C12" s="29" t="s">
+        <v>60</v>
       </c>
       <c r="D12" s="23"/>
       <c r="E12" s="23"/>
@@ -4706,8 +4649,8 @@
       <c r="J12" s="24"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="31" t="s">
-        <v>59</v>
+      <c r="A13" s="30" t="s">
+        <v>61</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -4733,7 +4676,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="22"/>
@@ -4771,7 +4714,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="22"/>
@@ -4785,7 +4728,7 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="15" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
@@ -4811,7 +4754,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="22"/>
@@ -5180,7 +5123,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1763127194" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1763650637" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5189,17 +5132,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
-  <drawing r:id="rId1"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763127194" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763650637" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5219,37 +5161,37 @@
   <sheetData>
     <row r="1" spans="5:19">
       <c r="E1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I1" s="25" t="n">
         <v>45950.9236111111095</v>
       </c>
       <c r="J1" s="25"/>
       <c r="O1" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -5261,28 +5203,28 @@
       <c r="I2" s="13"/>
       <c r="J2" s="13"/>
       <c r="O2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="8" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
@@ -5292,47 +5234,47 @@
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
       <c r="O3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="26" t="n">
-        <v>45975</v>
+        <v>45981</v>
       </c>
       <c r="D4" s="27"/>
       <c r="E4" s="28"/>
       <c r="F4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="S4" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -5341,27 +5283,27 @@
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="8" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
       <c r="S5" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="7" spans="1:10">
       <c r="A7" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -5375,40 +5317,40 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="8" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="9" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G9" s="11"/>
       <c r="H9" s="9" t="s">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
@@ -5416,7 +5358,7 @@
     <row r="10" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="11" spans="1:10">
       <c r="A11" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -5430,11 +5372,11 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="11"/>
-      <c r="C12" s="30" t="s">
-        <v>61</v>
+      <c r="C12" s="29" t="s">
+        <v>64</v>
       </c>
       <c r="D12" s="23"/>
       <c r="E12" s="23"/>
@@ -5445,8 +5387,8 @@
       <c r="J12" s="24"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="31" t="s">
-        <v>62</v>
+      <c r="A13" s="30" t="s">
+        <v>65</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -5472,7 +5414,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="22"/>
@@ -5510,7 +5452,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="22"/>
@@ -5524,7 +5466,7 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="15" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
@@ -5550,7 +5492,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="22"/>
@@ -5919,7 +5861,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1763127194" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1763650637" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -5928,16 +5870,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763127194" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763650637" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -5957,37 +5899,37 @@
   <sheetData>
     <row r="1" spans="5:19">
       <c r="E1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I1" s="25" t="n">
         <v>45950.9236111111095</v>
       </c>
       <c r="J1" s="25"/>
       <c r="O1" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -5999,28 +5941,28 @@
       <c r="I2" s="13"/>
       <c r="J2" s="13"/>
       <c r="O2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="8" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
@@ -6030,24 +5972,24 @@
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
       <c r="O3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="26" t="n">
@@ -6056,21 +5998,21 @@
       <c r="D4" s="27"/>
       <c r="E4" s="28"/>
       <c r="F4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="S4" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -6079,27 +6021,27 @@
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
       <c r="S5" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="7" spans="1:10">
       <c r="A7" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -6113,40 +6055,40 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="9" t="s">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="9" t="s">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G9" s="11"/>
       <c r="H9" s="9" t="s">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="I9" s="9"/>
       <c r="J9" s="9"/>
@@ -6154,7 +6096,7 @@
     <row r="10" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="11" spans="1:10">
       <c r="A11" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -6168,11 +6110,11 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="11"/>
-      <c r="C12" s="30" t="s">
-        <v>67</v>
+      <c r="C12" s="29" t="s">
+        <v>68</v>
       </c>
       <c r="D12" s="23"/>
       <c r="E12" s="23"/>
@@ -6183,8 +6125,8 @@
       <c r="J12" s="24"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="31" t="s">
-        <v>68</v>
+      <c r="A13" s="30" t="s">
+        <v>69</v>
       </c>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
@@ -6210,7 +6152,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="22"/>
@@ -6248,7 +6190,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="22"/>
@@ -6262,7 +6204,7 @@
     </row>
     <row r="19" spans="1:10">
       <c r="A19" s="15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B19" s="16"/>
       <c r="C19" s="16"/>
@@ -6288,7 +6230,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="22"/>
@@ -6657,7 +6599,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1763127194" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1763650637" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -6666,17 +6608,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
-  <drawing r:id="rId1"/>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763127194" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763650637" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -6696,37 +6637,37 @@
   <sheetData>
     <row r="1" spans="5:19">
       <c r="E1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I1" s="25" t="n">
         <v>45950.9236111111095</v>
       </c>
       <c r="J1" s="25"/>
       <c r="O1" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -6738,24 +6679,24 @@
       <c r="I2" s="13"/>
       <c r="J2" s="13"/>
       <c r="O2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="8"/>
@@ -6767,45 +6708,45 @@
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
       <c r="O3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="26"/>
       <c r="D4" s="27"/>
       <c r="E4" s="28"/>
       <c r="F4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="S4" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -6814,27 +6755,27 @@
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
       <c r="S5" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="7" spans="1:10">
       <c r="A7" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -6848,34 +6789,34 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="9" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G9" s="11"/>
       <c r="H9" s="9"/>
@@ -6885,7 +6826,7 @@
     <row r="10" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="11" spans="1:10">
       <c r="A11" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -6899,10 +6840,10 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="11"/>
-      <c r="C12" s="30"/>
+      <c r="C12" s="29"/>
       <c r="D12" s="23"/>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
@@ -6912,7 +6853,7 @@
       <c r="J12" s="24"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="31"/>
+      <c r="A13" s="30"/>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
@@ -6937,7 +6878,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="22"/>
@@ -6975,7 +6916,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="22"/>
@@ -7013,7 +6954,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="22"/>
@@ -7382,7 +7323,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1763127194" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1763650637" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -7391,16 +7332,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763127194" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763650637" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -7420,37 +7361,37 @@
   <sheetData>
     <row r="1" spans="5:19">
       <c r="E1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I1" s="25" t="n">
         <v>45950.9236111111095</v>
       </c>
       <c r="J1" s="25"/>
       <c r="O1" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -7462,24 +7403,24 @@
       <c r="I2" s="13"/>
       <c r="J2" s="13"/>
       <c r="O2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="8"/>
@@ -7491,31 +7432,31 @@
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
       <c r="O3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="26"/>
       <c r="D4" s="27"/>
       <c r="E4" s="28"/>
       <c r="F4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="8"/>
@@ -7523,11 +7464,11 @@
       <c r="J4" s="8"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="S4" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -7536,27 +7477,27 @@
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
       <c r="S5" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="7" spans="1:10">
       <c r="A7" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -7570,34 +7511,34 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="9" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G9" s="11"/>
       <c r="H9" s="9"/>
@@ -7607,7 +7548,7 @@
     <row r="10" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="11" spans="1:10">
       <c r="A11" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -7621,10 +7562,10 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="11"/>
-      <c r="C12" s="30"/>
+      <c r="C12" s="29"/>
       <c r="D12" s="23"/>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
@@ -7634,7 +7575,7 @@
       <c r="J12" s="24"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="31"/>
+      <c r="A13" s="30"/>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
@@ -7659,7 +7600,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="22"/>
@@ -7697,7 +7638,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="22"/>
@@ -7735,7 +7676,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="22"/>
@@ -8104,7 +8045,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1763127194" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1763650637" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -8113,16 +8054,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763127194" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763650637" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>
@@ -8142,37 +8083,37 @@
   <sheetData>
     <row r="1" spans="5:19">
       <c r="E1" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I1" s="25" t="n">
         <v>45950.9236111111095</v>
       </c>
       <c r="J1" s="25"/>
       <c r="O1" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P1" s="5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q1" s="5" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="R1" s="5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="S1" s="5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:19">
       <c r="A2" s="13" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
@@ -8184,24 +8125,24 @@
       <c r="I2" s="13"/>
       <c r="J2" s="13"/>
       <c r="O2" s="6" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="P2" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q2" s="6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="R2" s="6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="S2" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="8"/>
@@ -8213,45 +8154,45 @@
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
       <c r="O3" s="6" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="P3" s="6" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="Q3" s="6" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="R3" s="6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="S3" s="6" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="26"/>
       <c r="D4" s="27"/>
       <c r="E4" s="28"/>
       <c r="F4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
       <c r="O4" s="6"/>
       <c r="P4" s="6" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="Q4" s="6"/>
       <c r="S4" s="6" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:19">
@@ -8260,27 +8201,27 @@
       </c>
       <c r="B5" s="11"/>
       <c r="C5" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="11" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="8" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
       <c r="S5" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="7" spans="1:10">
       <c r="A7" s="13" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -8294,34 +8235,34 @@
     </row>
     <row r="8" spans="1:10">
       <c r="A8" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" s="11"/>
       <c r="C8" s="9" t="s">
-        <v>53</v>
+        <v>71</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G8" s="11"/>
       <c r="H8" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="8"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9" s="11" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B9" s="11"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
       <c r="E9" s="9"/>
       <c r="F9" s="11" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G9" s="11"/>
       <c r="H9" s="9"/>
@@ -8331,7 +8272,7 @@
     <row r="10" spans="1:1" ht="7.95" customHeight="1"/>
     <row r="11" spans="1:10">
       <c r="A11" s="13" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -8345,10 +8286,10 @@
     </row>
     <row r="12" spans="1:10">
       <c r="A12" s="11" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B12" s="11"/>
-      <c r="C12" s="30"/>
+      <c r="C12" s="29"/>
       <c r="D12" s="23"/>
       <c r="E12" s="23"/>
       <c r="F12" s="23"/>
@@ -8358,7 +8299,7 @@
       <c r="J12" s="24"/>
     </row>
     <row r="13" spans="1:10">
-      <c r="A13" s="31"/>
+      <c r="A13" s="30"/>
       <c r="B13" s="16"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
@@ -8383,7 +8324,7 @@
     </row>
     <row r="15" spans="1:10">
       <c r="A15" s="11" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B15" s="11"/>
       <c r="C15" s="22"/>
@@ -8421,7 +8362,7 @@
     </row>
     <row r="18" spans="1:10">
       <c r="A18" s="11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B18" s="11"/>
       <c r="C18" s="22"/>
@@ -8459,7 +8400,7 @@
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="11" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="11"/>
       <c r="C21" s="22"/>
@@ -8828,7 +8769,7 @@
   <printOptions>
     <extLst>
       <ext uri="smNativeData">
-        <pm:pageFlags xmlns:pm="smNativeData" id="1763127194" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
+        <pm:pageFlags xmlns:pm="smNativeData" id="1763650637" printRowHead="0" printColHead="0" printHeadLine="0" printFootLine="0" autoHeightHeader="0" autoHeightFooter="0" fitToPageBoth="0"/>
       </ext>
     </extLst>
   </printOptions>
@@ -8837,16 +8778,16 @@
   <headerFooter>
     <extLst>
       <ext uri="smNativeData">
-        <pm:header xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
-        <pm:footer xmlns:pm="smNativeData" id="1763127194" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="0" type="0" value="0"/>
-        <pm:paperBin xmlns:pm="smNativeData" id="1763127194" Id="1" type="0" value="0"/>
+        <pm:header xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="0"/>
+        <pm:footer xmlns:pm="smNativeData" id="1763650637" l="56" r="56" t="56" b="56" borderId="0" fillId="0" vertical="2"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="0" type="0" value="0"/>
+        <pm:paperBin xmlns:pm="smNativeData" id="1763650637" Id="1" type="0" value="0"/>
       </ext>
     </extLst>
   </headerFooter>
   <extLst>
     <ext uri="smNativeData">
-      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763127194" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
+      <pm:sheetPrefs xmlns:pm="smNativeData" day="1763650637" outlineProtect="1" showHorizontalRuler="1" showVerticalRuler="1" showAltShade="0">
         <pm:shade id="0" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
         <pm:shade id="1" type="0" fgLvl="100" fgClr="000000" bgLvl="100" bgClr="FFFFFF"/>
       </pm:sheetPrefs>

</xml_diff>